<commit_message>
Completed SNF analysis and report
</commit_message>
<xml_diff>
--- a/Results/single_algorithm/SNF/Supplement/Chisq_tests.xlsx
+++ b/Results/single_algorithm/SNF/Supplement/Chisq_tests.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
   <si>
     <t xml:space="preserve">Comparison</t>
   </si>
@@ -29,10 +29,10 @@
     <t xml:space="preserve">Vital status vs SNF cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.437116803424344</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.77636422427866</t>
+    <t xml:space="preserve">0.879669788483233</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.256417364580257</t>
   </si>
   <si>
     <t xml:space="preserve">0</t>
@@ -41,118 +41,112 @@
     <t xml:space="preserve">Ethnicity vs SNF cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.629146909688629</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.58689192487927</t>
+    <t xml:space="preserve">0.905006398288344</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.199626530750662</t>
   </si>
   <si>
     <t xml:space="preserve">Race vs SNF cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">6.26972828364888e-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">38.4296423817604</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.154</t>
+    <t xml:space="preserve">1.19386720959497e-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28.0937992733922</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.196</t>
   </si>
   <si>
     <t xml:space="preserve">Lymph node status vs SNF cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.014901450167854</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12.3544141260219</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.081</t>
+    <t xml:space="preserve">0.789786803096747</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.471984478880369</t>
   </si>
   <si>
     <t xml:space="preserve">Histology vs SNF cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">1.33432805116392e-19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">128.361784985076</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.296</t>
+    <t xml:space="preserve">4.78436363888453e-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">85.0033403826468</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.351</t>
   </si>
   <si>
     <t xml:space="preserve">Menopausal status vs SNF cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.329774898858886</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.1503135839159</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.03</t>
+    <t xml:space="preserve">0.137061126313304</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.97789252883777</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.069</t>
   </si>
   <si>
     <t xml:space="preserve">PR status vs SNF cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">5.14194633171403e-49</t>
-  </si>
-  <si>
-    <t xml:space="preserve">240.178428126942</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.427</t>
+    <t xml:space="preserve">1.5612862535955e-52</t>
+  </si>
+  <si>
+    <t xml:space="preserve">243.630057088538</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.621</t>
   </si>
   <si>
     <t xml:space="preserve">ER status vs SNF cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">4.76372983471144e-75</t>
-  </si>
-  <si>
-    <t xml:space="preserve">352.62150981006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.521</t>
+    <t xml:space="preserve">1.32447924336392e-70</t>
+  </si>
+  <si>
+    <t xml:space="preserve">321.799874302551</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.716</t>
   </si>
   <si>
     <t xml:space="preserve">HER2 status vs SNF cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.00383377884065525</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22.6569409703719</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.107</t>
+    <t xml:space="preserve">0.658314629560086</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.42388824966683</t>
   </si>
   <si>
     <t xml:space="preserve">Metastasis vs SNF cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.345543541506543</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.47482071335948</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.019</t>
+    <t xml:space="preserve">0.0692167532984767</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.34102469194189</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.073</t>
   </si>
   <si>
     <t xml:space="preserve">Stage vs SNF cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.0150750587731031</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18.9599961358455</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.092</t>
+    <t xml:space="preserve">0.0999417712292103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.7809047116105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.078</t>
   </si>
 </sst>
 </file>
@@ -548,105 +542,105 @@
         <v>17</v>
       </c>
       <c r="D5" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" t="s">
         <v>19</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>20</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>21</v>
-      </c>
-      <c r="D6" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" t="s">
         <v>23</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>24</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>25</v>
-      </c>
-      <c r="D7" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" t="s">
         <v>27</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>28</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>29</v>
-      </c>
-      <c r="D8" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" t="s">
         <v>31</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>32</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>33</v>
-      </c>
-      <c r="D9" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" t="s">
         <v>35</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>36</v>
       </c>
-      <c r="C10" t="s">
-        <v>37</v>
-      </c>
       <c r="D10" t="s">
-        <v>38</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" t="s">
         <v>39</v>
       </c>
-      <c r="B11" t="s">
+      <c r="D11" t="s">
         <v>40</v>
-      </c>
-      <c r="C11" t="s">
-        <v>41</v>
-      </c>
-      <c r="D11" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" t="s">
         <v>43</v>
       </c>
-      <c r="B12" t="s">
+      <c r="D12" t="s">
         <v>44</v>
-      </c>
-      <c r="C12" t="s">
-        <v>45</v>
-      </c>
-      <c r="D12" t="s">
-        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated individual SNF analysis
</commit_message>
<xml_diff>
--- a/Results/single_algorithm/SNF/Supplement/Chisq_tests.xlsx
+++ b/Results/single_algorithm/SNF/Supplement/Chisq_tests.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t xml:space="preserve">Comparison</t>
   </si>
@@ -29,10 +29,10 @@
     <t xml:space="preserve">Vital status vs SNF cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.879669788483233</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.256417364580257</t>
+    <t xml:space="preserve">0.999999999999999</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.53212544352703e-30</t>
   </si>
   <si>
     <t xml:space="preserve">0</t>
@@ -41,112 +41,109 @@
     <t xml:space="preserve">Ethnicity vs SNF cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.905006398288344</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.199626530750662</t>
+    <t xml:space="preserve">0.999999999999996</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.60851912031316e-29</t>
   </si>
   <si>
     <t xml:space="preserve">Race vs SNF cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">1.19386720959497e-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">28.0937992733922</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.196</t>
+    <t xml:space="preserve">4.32857406353017e-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27.6369086300188</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.201</t>
   </si>
   <si>
     <t xml:space="preserve">Lymph node status vs SNF cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.789786803096747</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.471984478880369</t>
+    <t xml:space="preserve">0.724210564224837</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.12449402316312</t>
   </si>
   <si>
     <t xml:space="preserve">Histology vs SNF cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">4.78436363888453e-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">85.0033403826468</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.351</t>
+    <t xml:space="preserve">5.9907772503684e-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">81.7720792674294</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.346</t>
   </si>
   <si>
     <t xml:space="preserve">Menopausal status vs SNF cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.137061126313304</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.97789252883777</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.069</t>
+    <t xml:space="preserve">0.0742799053651057</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.92643396299046</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.083</t>
   </si>
   <si>
     <t xml:space="preserve">PR status vs SNF cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">1.5612862535955e-52</t>
-  </si>
-  <si>
-    <t xml:space="preserve">243.630057088538</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.621</t>
+    <t xml:space="preserve">5.4291862013459e-54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">245.295611539606</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.645</t>
   </si>
   <si>
     <t xml:space="preserve">ER status vs SNF cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">1.32447924336392e-70</t>
-  </si>
-  <si>
-    <t xml:space="preserve">321.799874302551</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.716</t>
+    <t xml:space="preserve">2.88303346949335e-71</t>
+  </si>
+  <si>
+    <t xml:space="preserve">318.627563120099</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.741</t>
   </si>
   <si>
     <t xml:space="preserve">HER2 status vs SNF cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.658314629560086</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.42388824966683</t>
+    <t xml:space="preserve">0.536671396176457</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.17609928734168</t>
   </si>
   <si>
     <t xml:space="preserve">Metastasis vs SNF cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.0692167532984767</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.34102469194189</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.073</t>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.67913449601358e-31</t>
   </si>
   <si>
     <t xml:space="preserve">Stage vs SNF cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.0999417712292103</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.7809047116105</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.078</t>
+    <t xml:space="preserve">0.050748997674274</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.78154493926409</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.088</t>
   </si>
 </sst>
 </file>
@@ -626,21 +623,21 @@
         <v>39</v>
       </c>
       <c r="D11" t="s">
-        <v>40</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" t="s">
         <v>41</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>42</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>43</v>
-      </c>
-      <c r="D12" t="s">
-        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>